<commit_message>
Fix chart legends/axes; add plain-language walkthrough sheet to model
图 4/5/9/10 图例与坐标轴优化（图例移出数据区、年度刻度、标注避让）；
Excel 模型新增「说明-先看这页」工作表，逐步讲解七步计算。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01StQf2tSYTnPV9g2zDu1Bsq
</commit_message>
<xml_diff>
--- a/MT6102_Earnings_Model.xlsx
+++ b/MT6102_Earnings_Model.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Acquisition" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Earnings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="说明-先看这页" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Acquisition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Earnings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sensitivity" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="+#,##0;-#,##0;0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +63,16 @@
       <name val="Arial"/>
       <color rgb="00008000"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -98,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +126,18 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,6 +503,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr"/>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>这个表格怎么用（1 分钟看懂）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr"/>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>打开时如果数字是空白，按一下 F9 让 Excel 重算。蓝色字 = 可以改的输入；黄色格 = 情景开关；黑色字 = 自动算出来的，别动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="17" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>整个模型只有一条公式：年收益 = 每天租金 × 350 天 × 船数</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>350 天 = 一年 365 天减去 15 天维修检验（行业惯例）。租金全部用 Clarksons 上最近一笔真实成交，不是自己估的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="17" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>第1步</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>定每艘船的租金（见 Assumptions 表）：锁定的三艘 = 真实租约成交价（MR $30,000/天、Aframax $40,000/天、Kamsarmax $22,000/天）；跑现货的两艘按三种行情各设一个数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>第2步</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>算每艘船一年赚多少（见 Earnings 表 4-8 行）。例：MR #1 = 30,000 × 350 = $10,500,000；Aframax = 40,000 × 350 = $14,000,000。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>第3步</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>五艘加总（Earnings 第 9 行）。基准情形：30,000+27,000+40,000+22,000+23,000 = 142,000 $/天 × 350 = $49,700,000。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>第4步</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>除以本金得收益率（第 10 行）：49.7M ÷ 250M = 19.9%。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>第5步</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>换行情只换两艘现货船的租金（Assumptions 黄色格）：坏行情用 2025 年平均价 → $43.3M（17.3%）；好行情用现在的现货价 → $53.3M（21.3%）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>第6步</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>扣营运成本看净赚（第 12-14 行）：五艘每天共 36,560 美元（船员+保险+维修，Clarksons 官方数），×350 天 = $12.8M。净收益 = 49.7 − 12.8 = $36.9M（14.8%）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>第7步</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>敏感性（Sensitivity 表）：现货租金每变 1,000 美元/天，年收益变 2 艘 × 350 天 × 1,000 = 70 万美元。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="17" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>四张表对应关系：Assumptions=输入 | Acquisition=买船花了多少钱 | Earnings=第2-6步 | Sensitivity=第7步</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>数据出处：Clarksons SIN，2026-09-12 提取；每笔成交的船名和日期都写在 Assumptions 的备注列。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -716,7 +901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -961,7 +1146,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1208,7 +1393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>